<commit_message>
Update village feed (120h lookback)
</commit_message>
<xml_diff>
--- a/data/google_news_dedup_audit_07_0426_UTC.xlsx
+++ b/data/google_news_dedup_audit_07_0426_UTC.xlsx
@@ -469,7 +469,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" t="n">
         <v>0.7187126874923706</v>
@@ -490,10 +490,10 @@
         <v>7</v>
       </c>
       <c r="B4" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6037429571151733</v>
+        <v>0.5831209421157837</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -502,19 +502,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Amazon US Portal Deal: Amazon and USPS Finalize Major Delivery Partnership - Meyka</t>
+          <t>Amazon and USPS Seal Landmark Delivery Deal - Devdiscourse</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9484189748764038</v>
+        <v>0.7006281614303589</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -523,19 +523,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Amazon reaches delivery agreement with U.S. Postal Service - Investing.com</t>
+          <t>Amazon Reaches US Postal Service Deal for 1 Billion Packages - Bloomberg.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8694539666175842</v>
+        <v>0.9484189748764038</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -544,19 +544,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Amazon reaches delivery agreement with U.S. Postal Service By Investing.com - Investing.com Canada</t>
+          <t>Amazon reaches delivery agreement with U.S. Postal Service - Investing.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7006281614303589</v>
+        <v>0.8694539666175842</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -565,16 +565,16 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Amazon Reaches US Postal Service Deal for 1 Billion Packages - Bloomberg.com</t>
+          <t>Amazon reaches delivery agreement with U.S. Postal Service By Investing.com - Investing.com Canada</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C8" t="n">
         <v>0.7178592681884766</v>
@@ -592,76 +592,76 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7032829523086548</v>
+        <v>0.8196215629577637</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FedEx, Amazon up race for faster delivery - MSN</t>
+          <t>Amazon launches new way to order UberEats, Grubhub with Alexa: ‘Same way you would with a waiter’ - New York Post</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FedEx's same-day delivery rollout is more about optionality than speed - MSN</t>
+          <t>Food Delivery, Including Grubhub and Uber Eats, Comes to Amazon’s Alexa+ - People.com</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B10" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8196215629577637</v>
+        <v>0.7952001094818115</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Amazon launches new way to order UberEats, Grubhub with Alexa: ‘Same way you would with a waiter’ - New York Post</t>
+          <t>M&amp;S calls for crackdown on ‘brazen, organised, aggressive’ retail crime | Marks &amp; Spencer - The Guardian</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Food Delivery, Including Grubhub and Uber Eats, Comes to Amazon’s Alexa+ - People.com</t>
+          <t>Marks &amp; Spencer warns retail crime is spiralling as shoplifting turns organised and violent - EasternEye</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B11" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7952001094818115</v>
+        <v>0.6921748518943787</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>M&amp;S calls for crackdown on ‘brazen, organised, aggressive’ retail crime | Marks &amp; Spencer - The Guardian</t>
+          <t>Man in levensgevaar na steekpartij in stationsbuurt Antwerpen - VRT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Marks &amp; Spencer warns retail crime is spiralling as shoplifting turns organised and violent - EasternEye</t>
+          <t>Beelden tonen vechtpartij waarbij jongeman levensgevaarlijk gewond raakt in Carnotstraat in Antwerpen - HLN</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C12" t="n">
-        <v>0.6921748518943787</v>
+        <v>0.7059022784233093</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -670,19 +670,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Beelden tonen vechtpartij waarbij jongeman levensgevaarlijk gewond raakt in Carnotstraat in Antwerpen - HLN</t>
+          <t>Twee gewonden bij steekpartij in Antwerpse Carnotstraat, één slachtoffer in levensgevaar: “Gebeurt wel vaker” - GVA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C13" t="n">
-        <v>0.7059022784233093</v>
+        <v>0.6814751625061035</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -691,19 +691,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Twee gewonden bij steekpartij in Antwerpse Carnotstraat, één slachtoffer in levensgevaar: “Gebeurt wel vaker” - GVA</t>
+          <t>Twee gewonden bij steekpartij in Antwerpse Carnotstraat, één slachtoffer in levensgevaar: “Gebeurt wel vaker” - Nieuwsblad</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B14" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C14" t="n">
-        <v>0.6814751625061035</v>
+        <v>0.9722259044647217</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -712,19 +712,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Twee gewonden bij steekpartij in Antwerpse Carnotstraat, één slachtoffer in levensgevaar: “Gebeurt wel vaker” - Nieuwsblad</t>
+          <t>Man in levensgevaar na steekpartij in stationsbuurt Antwerpen - v-nieuws</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B15" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9722259044647217</v>
+        <v>0.6507700681686401</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -733,19 +733,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Man in levensgevaar na steekpartij in stationsbuurt Antwerpen - v-nieuws</t>
+          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen | Foto - HLN</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C16" t="n">
-        <v>0.6507700681686401</v>
+        <v>0.6528626680374146</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -754,19 +754,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen | Foto - HLN</t>
+          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen | Foto - pzc.nl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B17" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C17" t="n">
-        <v>0.6528626680374146</v>
+        <v>0.6796237230300903</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -775,19 +775,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen | Foto - pzc.nl</t>
+          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen - HLN</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B18" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C18" t="n">
-        <v>0.6796236634254456</v>
+        <v>0.6507700681686401</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -796,19 +796,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen - HLN</t>
+          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen | Foto - HLN</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B19" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C19" t="n">
-        <v>0.6507700681686401</v>
+        <v>0.6542749404907227</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -817,19 +817,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Slachtoffer in levensgevaar na steekpartij in Carnotstraat in Antwerpen | Foto - HLN</t>
+          <t>Beelden tonen vechtpartij waarbij jongeman levensgevaarlijk gewond raakt in Carnotstraat in Antwerpen | Foto - HLN</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B20" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C20" t="n">
-        <v>0.6542749404907227</v>
+        <v>0.6512234210968018</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -838,19 +838,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Beelden tonen vechtpartij waarbij jongeman levensgevaarlijk gewond raakt in Carnotstraat in Antwerpen | Foto - HLN</t>
+          <t>Beelden van vechtpartij in Antwerpen - HLN</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B21" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C21" t="n">
-        <v>0.6512234210968018</v>
+        <v>0.9285715818405151</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -859,16 +859,16 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Beelden van vechtpartij in Antwerpen - HLN</t>
+          <t>Man in levensgevaar bij steekpartij in Antwerpse stationsbuurt - msn.com</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B22" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="C22" t="n">
         <v>0.7079473733901978</v>
@@ -886,52 +886,52 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B23" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C23" t="n">
-        <v>0.9977073669433594</v>
+        <v>0.9973177909851074</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Assises à Anvers - Said Cherkaoui condamné à la prison à perpétuité pour l'assassinat de Davy Veraghtert - msn.com</t>
+          <t>Assises à Anvers - Said Cherkaoui condamné à la prison à perpétuité pour l'assassinat de Davy Veraghtert - MSN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Assises Anvers - Said Cherkaoui condamné à la prison à perpétuité pour l'assassinat de Davy Veraghtert - msn.com</t>
+          <t>Assises Anvers - Said Cherkaoui condamné à la prison à perpétuité pour l'assassinat de Davy Veraghtert - MSN</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B24" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C24" t="n">
-        <v>0.7597138285636902</v>
+        <v>0.772411584854126</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Assises à Anvers - Said Cherkaoui condamné à la prison à perpétuité pour l'assassinat de Davy Veraghtert - msn.com</t>
+          <t>Assises à Anvers - Said Cherkaoui condamné à la prison à perpétuité pour l'assassinat de Davy Veraghtert - MSN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Assises Anvers - Said Cherkaoui reconnu coupable de l'assassinat de Davy Veraghtert - msn.com</t>
+          <t>Assises Anvers - Said Cherkaoui reconnu coupable de l'assassinat de Davy Veraghtert - MSN</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B25" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C25" t="n">
         <v>0.839720606803894</v>
@@ -949,10 +949,10 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B26" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C26" t="n">
         <v>0.7169114351272583</v>
@@ -970,10 +970,10 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B27" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C27" t="n">
         <v>0.8102166652679443</v>
@@ -991,13 +991,13 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B28" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C28" t="n">
-        <v>0.8166295289993286</v>
+        <v>0.8224859833717346</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1006,16 +1006,16 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Teen Stuck In Freezing Mud Rescued From Wertheim National Wildlife Refuge In Shirley: Police - Patch</t>
+          <t>Teen Stuck In Freezing Mud Rescued From Wertheim National Wildlife Refuge In Shirley: Police - patch.com</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B29" t="n">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C29" t="n">
         <v>0.7251365780830383</v>
@@ -1033,10 +1033,10 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B30" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C30" t="n">
         <v>0.8023912310600281</v>
@@ -1054,10 +1054,10 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B31" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C31" t="n">
         <v>0.8328729867935181</v>
@@ -1075,10 +1075,10 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B32" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C32" t="n">
         <v>0.7582589387893677</v>
@@ -1096,10 +1096,10 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B33" t="n">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C33" t="n">
         <v>0.5874330997467041</v>
@@ -1117,10 +1117,10 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B34" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C34" t="n">
         <v>0.7055689096450806</v>
@@ -1138,10 +1138,10 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B35" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C35" t="n">
         <v>0.6020748615264893</v>
@@ -1159,10 +1159,10 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B36" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C36" t="n">
         <v>0.6221848130226135</v>
@@ -1180,10 +1180,10 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B37" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C37" t="n">
         <v>0.7280769348144531</v>
@@ -1201,38 +1201,38 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B38" t="n">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C38" t="n">
         <v>0.7047463655471802</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
+          <t>LIVE as man stabbed to death and two fighting for life after Peckham stabbing - London Now</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
           <t>Two men fighting for their lives after triple stabbing in south east London - Yahoo News UK</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>LIVE as man stabbed to death and two fighting for life after Peckham stabbing - London Now</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B39" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C39" t="n">
-        <v>0.631381630897522</v>
+        <v>0.8538622856140137</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Two men fighting for their lives after triple stabbing in south east London - Yahoo News UK</t>
+          <t>LIVE as man stabbed to death and two fighting for life after Peckham stabbing - London Now</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1243,17 +1243,17 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B40" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C40" t="n">
-        <v>0.9660229682922363</v>
+        <v>0.735625147819519</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Two men fighting for their lives after triple stabbing in south east London - Yahoo News UK</t>
+          <t>LIVE as man stabbed to death and two fighting for life after Peckham stabbing - London Now</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1264,52 +1264,52 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B41" t="n">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C41" t="n">
-        <v>0.7726439237594604</v>
+        <v>0.9999998807907104</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Two more people arrested on suspicion of murder after 14-year-old boy shot dead in London - Sky News</t>
+          <t>Investing in America: 1937 New London Explosion - KETK.com</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Two more murder arrests over shooting of 14-year-old in London | News - Hits Radio - Rayo</t>
+          <t>Investing in America: 1937 New London Explosion - KETK.com</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B42" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C42" t="n">
-        <v>0.9999998211860657</v>
+        <v>0.7880639433860779</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Investing in America: 1937 New London Explosion - KETK.com</t>
+          <t>Two more people arrested on suspicion of murder after 14-year-old boy shot dead in London - Sky News</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Investing in America: 1937 New London Explosion - KETK.com</t>
+          <t>Two more murder arrests over shooting of 14-year-old in London | News - Hits Radio - planetradio.co.uk</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B43" t="n">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C43" t="n">
         <v>0.7339832782745361</v>
@@ -1327,13 +1327,13 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="B44" t="n">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="C44" t="n">
-        <v>0.7738058567047119</v>
+        <v>0.7738057374954224</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="B45" t="n">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="C45" t="n">
         <v>0.663328230381012</v>
@@ -1369,10 +1369,10 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="B46" t="n">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="C46" t="n">
         <v>0.7277822494506836</v>
@@ -1390,10 +1390,10 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="B47" t="n">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="C47" t="n">
         <v>0.7065956592559814</v>

</xml_diff>